<commit_message>
Release v3 UI and retry flow
</commit_message>
<xml_diff>
--- a/voci.xlsx
+++ b/voci.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniekonig/Local_Documents/codex_projects/voci/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B254B3-D3C4-0F4D-9158-F4D97E19B880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007BB097-68E7-1E49-971F-BB4D70713E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="580" windowWidth="28040" windowHeight="17000" xr2:uid="{BDCBCED7-AD98-464C-B035-406A12369206}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>DE</t>
   </si>
@@ -66,6 +66,12 @@
   </si>
   <si>
     <t>vier</t>
+  </si>
+  <si>
+    <t>Haus</t>
+  </si>
+  <si>
+    <t>house</t>
   </si>
 </sst>
 </file>
@@ -437,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F6005F0-BBA9-244F-8C1F-31795C012788}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -478,6 +484,14 @@
       </c>
       <c r="B5" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improve wrong answer feedback
</commit_message>
<xml_diff>
--- a/voci.xlsx
+++ b/voci.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniekonig/Local_Documents/codex_projects/voci/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007BB097-68E7-1E49-971F-BB4D70713E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9919FDDA-D308-8149-A83E-74D5373EAB8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="580" windowWidth="28040" windowHeight="17000" xr2:uid="{BDCBCED7-AD98-464C-B035-406A12369206}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>DE</t>
   </si>
@@ -72,6 +72,27 @@
   </si>
   <si>
     <t>house</t>
+  </si>
+  <si>
+    <t>Maus</t>
+  </si>
+  <si>
+    <t>mouse</t>
+  </si>
+  <si>
+    <t>Katze</t>
+  </si>
+  <si>
+    <t>cat</t>
+  </si>
+  <si>
+    <t>Hund</t>
+  </si>
+  <si>
+    <t>dog</t>
+  </si>
+  <si>
+    <t>Wie viele Kantone zählt die Schweiz?</t>
   </si>
 </sst>
 </file>
@@ -443,8 +464,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F6005F0-BBA9-244F-8C1F-31795C012788}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -492,6 +516,38 @@
       </c>
       <c r="B6" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add multi-list sheet selection
</commit_message>
<xml_diff>
--- a/voci.xlsx
+++ b/voci.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniekonig/Local_Documents/codex_projects/voci/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9919FDDA-D308-8149-A83E-74D5373EAB8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D07ECC3-0F0E-9946-AC3E-DFDE7241DC8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="580" windowWidth="28040" windowHeight="17000" xr2:uid="{BDCBCED7-AD98-464C-B035-406A12369206}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="28800" windowHeight="18060" activeTab="2" xr2:uid="{BDCBCED7-AD98-464C-B035-406A12369206}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Liste 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Liste 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Liste 3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
   <si>
     <t>DE</t>
   </si>
@@ -93,6 +95,30 @@
   </si>
   <si>
     <t>Wie viele Kantone zählt die Schweiz?</t>
+  </si>
+  <si>
+    <t>sechs</t>
+  </si>
+  <si>
+    <t>six</t>
+  </si>
+  <si>
+    <t>sieben</t>
+  </si>
+  <si>
+    <t>seven</t>
+  </si>
+  <si>
+    <t>acht</t>
+  </si>
+  <si>
+    <t>eight</t>
+  </si>
+  <si>
+    <t>neun</t>
+  </si>
+  <si>
+    <t>nine</t>
   </si>
 </sst>
 </file>
@@ -554,4 +580,72 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AB7ABE5-9F69-6642-91F3-7B9F916D9774}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DC6CEA-05A5-F54B-8D9B-9B276DA9F849}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add word subselection per list
</commit_message>
<xml_diff>
--- a/voci.xlsx
+++ b/voci.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniekonig/Local_Documents/codex_projects/voci/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D07ECC3-0F0E-9946-AC3E-DFDE7241DC8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD20DE0E-C41D-484C-BBD3-B40120468806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="28800" windowHeight="18060" activeTab="2" xr2:uid="{BDCBCED7-AD98-464C-B035-406A12369206}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="28800" windowHeight="18060" activeTab="3" xr2:uid="{BDCBCED7-AD98-464C-B035-406A12369206}"/>
   </bookViews>
   <sheets>
-    <sheet name="Liste 1" sheetId="1" r:id="rId1"/>
-    <sheet name="Liste 2" sheetId="2" r:id="rId2"/>
-    <sheet name="Liste 3" sheetId="3" r:id="rId3"/>
+    <sheet name="English" sheetId="1" r:id="rId1"/>
+    <sheet name="NMG" sheetId="4" r:id="rId2"/>
+    <sheet name="numbers " sheetId="2" r:id="rId3"/>
+    <sheet name="more numbers" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
   <si>
     <t>DE</t>
   </si>
@@ -125,10 +126,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -154,8 +162,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,90 +499,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F6005F0-BBA9-244F-8C1F-31795C012788}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -583,15 +552,42 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AB7ABE5-9F69-6642-91F3-7B9F916D9774}">
-  <dimension ref="A1:B3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{297ACB97-01DA-1846-A44D-7BA679C70A5E}">
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AB7ABE5-9F69-6642-91F3-7B9F916D9774}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
@@ -609,6 +605,38 @@
       </c>
       <c r="B3" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -616,16 +644,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DC6CEA-05A5-F54B-8D9B-9B276DA9F849}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Compact layout and support Fragen Antworten headers
</commit_message>
<xml_diff>
--- a/voci.xlsx
+++ b/voci.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stephaniekonig/Local_Documents/codex_projects/voci/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD20DE0E-C41D-484C-BBD3-B40120468806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75B15CED-B87A-5B49-8217-E6B2C6C3CDAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="28800" windowHeight="18060" activeTab="3" xr2:uid="{BDCBCED7-AD98-464C-B035-406A12369206}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="28800" windowHeight="18060" activeTab="1" xr2:uid="{BDCBCED7-AD98-464C-B035-406A12369206}"/>
   </bookViews>
   <sheets>
     <sheet name="English" sheetId="1" r:id="rId1"/>
@@ -39,13 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
-  <si>
-    <t>DE</t>
-  </si>
-  <si>
-    <t>EN</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
   <si>
     <t>ein</t>
   </si>
@@ -120,6 +114,24 @@
   </si>
   <si>
     <t>nine</t>
+  </si>
+  <si>
+    <t>Fragen</t>
+  </si>
+  <si>
+    <t>Antworten</t>
+  </si>
+  <si>
+    <t>Der grösste See der Schwiez?</t>
+  </si>
+  <si>
+    <t>Lac de Néchatel</t>
+  </si>
+  <si>
+    <t>Der tiefste Punkt der Schwiez?</t>
+  </si>
+  <si>
+    <t>Lago Maggiore, 193M.ü.M</t>
   </si>
 </sst>
 </file>
@@ -507,42 +519,42 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -553,23 +565,43 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{297ACB97-01DA-1846-A44D-7BA679C70A5E}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2">
         <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -585,58 +617,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -651,29 +683,30 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>